<commit_message>
Update data anomali: 5 Juli 2026 pukul 10.59 WITA
</commit_message>
<xml_diff>
--- a/data/anomali/agregat_anomali_keluarga_per_kecamatan.xlsx
+++ b/data/anomali/agregat_anomali_keluarga_per_kecamatan.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="137">
   <si>
     <t>DATA RADAR ANOMALI KELUARGA</t>
   </si>
   <si>
-    <t>Seluruh data sampai Kecamatan | Dicetak: 30 Jun 2026, 06.30</t>
+    <t>Seluruh data sampai Kecamatan | Dicetak: 5 Jul 2026, 10.57</t>
   </si>
   <si>
     <t>Kode</t>
@@ -214,10 +214,16 @@
     <t>0</t>
   </si>
   <si>
-    <t>1,27</t>
-  </si>
-  <si>
-    <t>98,73</t>
+    <t>0,36</t>
+  </si>
+  <si>
+    <t>0,6</t>
+  </si>
+  <si>
+    <t>26,96</t>
+  </si>
+  <si>
+    <t>72,07</t>
   </si>
   <si>
     <t>7103</t>
@@ -232,10 +238,10 @@
     <t>MANGANITU SELATAN</t>
   </si>
   <si>
-    <t>0,24</t>
-  </si>
-  <si>
-    <t>99,76</t>
+    <t>63,41</t>
+  </si>
+  <si>
+    <t>36,59</t>
   </si>
   <si>
     <t>7103041</t>
@@ -244,121 +250,136 @@
     <t>TATOARENG</t>
   </si>
   <si>
+    <t>67,74</t>
+  </si>
+  <si>
+    <t>32,26</t>
+  </si>
+  <si>
+    <t>7103050</t>
+  </si>
+  <si>
+    <t>TAMAKO</t>
+  </si>
+  <si>
+    <t>2,5</t>
+  </si>
+  <si>
+    <t>97,5</t>
+  </si>
+  <si>
+    <t>7103060</t>
+  </si>
+  <si>
+    <t>TABUKAN SELATAN</t>
+  </si>
+  <si>
+    <t>20,34</t>
+  </si>
+  <si>
+    <t>79,66</t>
+  </si>
+  <si>
+    <t>7103061</t>
+  </si>
+  <si>
+    <t>TABUKAN SELATAN TENGAH</t>
+  </si>
+  <si>
+    <t>38,46</t>
+  </si>
+  <si>
+    <t>61,54</t>
+  </si>
+  <si>
+    <t>7103062</t>
+  </si>
+  <si>
+    <t>TABUKAN SELATAN TENGGARA</t>
+  </si>
+  <si>
+    <t>5,88</t>
+  </si>
+  <si>
+    <t>94,12</t>
+  </si>
+  <si>
+    <t>7103070</t>
+  </si>
+  <si>
+    <t>TABUKAN TENGAH</t>
+  </si>
+  <si>
+    <t>0,95</t>
+  </si>
+  <si>
+    <t>43,81</t>
+  </si>
+  <si>
+    <t>55,24</t>
+  </si>
+  <si>
+    <t>7103080</t>
+  </si>
+  <si>
+    <t>MANGANITU</t>
+  </si>
+  <si>
+    <t>3,33</t>
+  </si>
+  <si>
+    <t>96,67</t>
+  </si>
+  <si>
+    <t>7103090</t>
+  </si>
+  <si>
+    <t>TAHUNA</t>
+  </si>
+  <si>
+    <t>1,45</t>
+  </si>
+  <si>
+    <t>26,09</t>
+  </si>
+  <si>
+    <t>72,46</t>
+  </si>
+  <si>
+    <t>7103091</t>
+  </si>
+  <si>
+    <t>TAHUNA TIMUR</t>
+  </si>
+  <si>
+    <t>35,79</t>
+  </si>
+  <si>
+    <t>64,21</t>
+  </si>
+  <si>
+    <t>7103092</t>
+  </si>
+  <si>
+    <t>TAHUNA BARAT</t>
+  </si>
+  <si>
     <t>100</t>
   </si>
   <si>
-    <t>7103050</t>
-  </si>
-  <si>
-    <t>TAMAKO</t>
-  </si>
-  <si>
-    <t>0,89</t>
-  </si>
-  <si>
-    <t>99,11</t>
-  </si>
-  <si>
-    <t>7103060</t>
-  </si>
-  <si>
-    <t>TABUKAN SELATAN</t>
-  </si>
-  <si>
-    <t>0,44</t>
-  </si>
-  <si>
-    <t>99,56</t>
-  </si>
-  <si>
-    <t>7103061</t>
-  </si>
-  <si>
-    <t>TABUKAN SELATAN TENGAH</t>
-  </si>
-  <si>
-    <t>2,02</t>
-  </si>
-  <si>
-    <t>97,98</t>
-  </si>
-  <si>
-    <t>7103062</t>
-  </si>
-  <si>
-    <t>TABUKAN SELATAN TENGGARA</t>
-  </si>
-  <si>
-    <t>7103070</t>
-  </si>
-  <si>
-    <t>TABUKAN TENGAH</t>
-  </si>
-  <si>
-    <t>0,84</t>
-  </si>
-  <si>
-    <t>99,16</t>
-  </si>
-  <si>
-    <t>7103080</t>
-  </si>
-  <si>
-    <t>MANGANITU</t>
-  </si>
-  <si>
-    <t>2,49</t>
-  </si>
-  <si>
-    <t>97,51</t>
-  </si>
-  <si>
-    <t>7103090</t>
-  </si>
-  <si>
-    <t>TAHUNA</t>
-  </si>
-  <si>
-    <t>2,96</t>
-  </si>
-  <si>
-    <t>97,04</t>
-  </si>
-  <si>
-    <t>7103091</t>
-  </si>
-  <si>
-    <t>TAHUNA TIMUR</t>
-  </si>
-  <si>
-    <t>1,24</t>
-  </si>
-  <si>
-    <t>98,76</t>
-  </si>
-  <si>
-    <t>7103092</t>
-  </si>
-  <si>
-    <t>TAHUNA BARAT</t>
-  </si>
-  <si>
-    <t>2,07</t>
-  </si>
-  <si>
-    <t>97,93</t>
-  </si>
-  <si>
     <t>7103100</t>
   </si>
   <si>
     <t>TABUKAN UTARA</t>
   </si>
   <si>
-    <t>1,51</t>
-  </si>
-  <si>
-    <t>98,49</t>
+    <t>0,63</t>
+  </si>
+  <si>
+    <t>1,89</t>
+  </si>
+  <si>
+    <t>95,6</t>
   </si>
   <si>
     <t>7103101</t>
@@ -367,22 +388,34 @@
     <t>NUSA TABUKAN</t>
   </si>
   <si>
+    <t>11,11</t>
+  </si>
+  <si>
+    <t>88,89</t>
+  </si>
+  <si>
     <t>7103102</t>
   </si>
   <si>
     <t>KEPULAUAN MARORE</t>
   </si>
   <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
     <t>7103110</t>
   </si>
   <si>
     <t>KENDAHE</t>
   </si>
   <si>
-    <t>0,66</t>
-  </si>
-  <si>
-    <t>99,34</t>
+    <t>51,46</t>
+  </si>
+  <si>
+    <t>48,54</t>
   </si>
   <si>
     <t/>
@@ -1216,7 +1249,7 @@
         <v>65</v>
       </c>
       <c r="C6" s="7">
-        <v>11782</v>
+        <v>827</v>
       </c>
       <c r="D6" s="7">
         <v>0</v>
@@ -1243,10 +1276,10 @@
         <v>66</v>
       </c>
       <c r="L6" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M6" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N6" s="7">
         <v>0</v>
@@ -1255,10 +1288,10 @@
         <v>66</v>
       </c>
       <c r="P6" s="7">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R6" s="7">
         <v>0</v>
@@ -1267,10 +1300,10 @@
         <v>66</v>
       </c>
       <c r="T6" s="7">
-        <v>11632</v>
+        <v>223</v>
       </c>
       <c r="U6" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V6" s="7">
         <v>0</v>
@@ -1279,10 +1312,10 @@
         <v>66</v>
       </c>
       <c r="X6" s="7">
-        <v>0</v>
+        <v>596</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Z6" s="7">
         <v>0</v>
@@ -1305,79 +1338,79 @@
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="7">
+        <v>827</v>
+      </c>
+      <c r="D7" s="7">
+        <v>0</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="7">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="7">
+        <v>0</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="J7" s="7">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="L7" s="7">
+        <v>3</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="N7" s="7">
+        <v>0</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="P7" s="7">
+        <v>5</v>
+      </c>
+      <c r="Q7" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="R7" s="7">
+        <v>0</v>
+      </c>
+      <c r="S7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="T7" s="7">
+        <v>223</v>
+      </c>
+      <c r="U7" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="V7" s="7">
+        <v>0</v>
+      </c>
+      <c r="W7" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="X7" s="7">
+        <v>596</v>
+      </c>
+      <c r="Y7" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="C7" s="7">
-        <v>11782</v>
-      </c>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="F7" s="7">
-        <v>0</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="H7" s="7">
-        <v>0</v>
-      </c>
-      <c r="I7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" s="7">
-        <v>0</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="L7" s="7">
-        <v>0</v>
-      </c>
-      <c r="M7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="N7" s="7">
-        <v>0</v>
-      </c>
-      <c r="O7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="P7" s="7">
-        <v>150</v>
-      </c>
-      <c r="Q7" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="R7" s="7">
-        <v>0</v>
-      </c>
-      <c r="S7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="T7" s="7">
-        <v>11632</v>
-      </c>
-      <c r="U7" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="V7" s="7">
-        <v>0</v>
-      </c>
-      <c r="W7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="X7" s="7">
-        <v>0</v>
-      </c>
-      <c r="Y7" s="8" t="s">
-        <v>66</v>
       </c>
       <c r="Z7" s="7">
         <v>0</v>
@@ -1400,13 +1433,13 @@
     </row>
     <row r="8" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C8" s="10">
-        <v>1642</v>
+        <v>41</v>
       </c>
       <c r="D8" s="10">
         <v>0</v>
@@ -1445,10 +1478,10 @@
         <v>66</v>
       </c>
       <c r="P8" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="11" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="R8" s="10">
         <v>0</v>
@@ -1457,10 +1490,10 @@
         <v>66</v>
       </c>
       <c r="T8" s="10">
-        <v>1638</v>
+        <v>26</v>
       </c>
       <c r="U8" s="11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V8" s="10">
         <v>0</v>
@@ -1469,10 +1502,10 @@
         <v>66</v>
       </c>
       <c r="X8" s="10">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="Y8" s="11" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="Z8" s="10">
         <v>0</v>
@@ -1495,13 +1528,13 @@
     </row>
     <row r="9" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C9" s="10">
-        <v>312</v>
+        <v>31</v>
       </c>
       <c r="D9" s="10">
         <v>0</v>
@@ -1552,10 +1585,10 @@
         <v>66</v>
       </c>
       <c r="T9" s="10">
-        <v>312</v>
+        <v>21</v>
       </c>
       <c r="U9" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="V9" s="10">
         <v>0</v>
@@ -1564,10 +1597,10 @@
         <v>66</v>
       </c>
       <c r="X9" s="10">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Y9" s="11" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="Z9" s="10">
         <v>0</v>
@@ -1590,13 +1623,13 @@
     </row>
     <row r="10" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C10" s="10">
-        <v>1123</v>
+        <v>40</v>
       </c>
       <c r="D10" s="10">
         <v>0</v>
@@ -1635,10 +1668,10 @@
         <v>66</v>
       </c>
       <c r="P10" s="10">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="11" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="R10" s="10">
         <v>0</v>
@@ -1647,10 +1680,10 @@
         <v>66</v>
       </c>
       <c r="T10" s="10">
-        <v>1113</v>
+        <v>1</v>
       </c>
       <c r="U10" s="11" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="V10" s="10">
         <v>0</v>
@@ -1659,10 +1692,10 @@
         <v>66</v>
       </c>
       <c r="X10" s="10">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="Y10" s="11" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="Z10" s="10">
         <v>0</v>
@@ -1685,13 +1718,13 @@
     </row>
     <row r="11" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C11" s="10">
-        <v>915</v>
+        <v>59</v>
       </c>
       <c r="D11" s="10">
         <v>0</v>
@@ -1730,10 +1763,10 @@
         <v>66</v>
       </c>
       <c r="P11" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="11" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="R11" s="10">
         <v>0</v>
@@ -1742,10 +1775,10 @@
         <v>66</v>
       </c>
       <c r="T11" s="10">
-        <v>911</v>
+        <v>12</v>
       </c>
       <c r="U11" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="V11" s="10">
         <v>0</v>
@@ -1754,10 +1787,10 @@
         <v>66</v>
       </c>
       <c r="X11" s="10">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="Y11" s="11" t="s">
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="Z11" s="10">
         <v>0</v>
@@ -1780,13 +1813,13 @@
     </row>
     <row r="12" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C12" s="10">
-        <v>248</v>
+        <v>13</v>
       </c>
       <c r="D12" s="10">
         <v>0</v>
@@ -1825,22 +1858,22 @@
         <v>66</v>
       </c>
       <c r="P12" s="10">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="R12" s="10">
+        <v>0</v>
+      </c>
+      <c r="S12" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="T12" s="10">
         <v>5</v>
       </c>
-      <c r="Q12" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="R12" s="10">
-        <v>0</v>
-      </c>
-      <c r="S12" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="T12" s="10">
-        <v>243</v>
-      </c>
       <c r="U12" s="11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="V12" s="10">
         <v>0</v>
@@ -1849,10 +1882,10 @@
         <v>66</v>
       </c>
       <c r="X12" s="10">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Y12" s="11" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="Z12" s="10">
         <v>0</v>
@@ -1875,13 +1908,13 @@
     </row>
     <row r="13" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C13" s="10">
-        <v>272</v>
+        <v>17</v>
       </c>
       <c r="D13" s="10">
         <v>0</v>
@@ -1932,10 +1965,10 @@
         <v>66</v>
       </c>
       <c r="T13" s="10">
-        <v>272</v>
+        <v>1</v>
       </c>
       <c r="U13" s="11" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="V13" s="10">
         <v>0</v>
@@ -1944,10 +1977,10 @@
         <v>66</v>
       </c>
       <c r="X13" s="10">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Y13" s="11" t="s">
-        <v>66</v>
+        <v>96</v>
       </c>
       <c r="Z13" s="10">
         <v>0</v>
@@ -1970,13 +2003,13 @@
     </row>
     <row r="14" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C14" s="10">
-        <v>947</v>
+        <v>105</v>
       </c>
       <c r="D14" s="10">
         <v>0</v>
@@ -2015,10 +2048,10 @@
         <v>66</v>
       </c>
       <c r="P14" s="10">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="Q14" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="R14" s="10">
         <v>0</v>
@@ -2027,10 +2060,10 @@
         <v>66</v>
       </c>
       <c r="T14" s="10">
-        <v>939</v>
+        <v>46</v>
       </c>
       <c r="U14" s="11" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="V14" s="10">
         <v>0</v>
@@ -2039,10 +2072,10 @@
         <v>66</v>
       </c>
       <c r="X14" s="10">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="Y14" s="11" t="s">
-        <v>66</v>
+        <v>101</v>
       </c>
       <c r="Z14" s="10">
         <v>0</v>
@@ -2065,13 +2098,13 @@
     </row>
     <row r="15" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C15" s="10">
-        <v>962</v>
+        <v>60</v>
       </c>
       <c r="D15" s="10">
         <v>0</v>
@@ -2110,10 +2143,10 @@
         <v>66</v>
       </c>
       <c r="P15" s="10">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="11" t="s">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="R15" s="10">
         <v>0</v>
@@ -2122,10 +2155,10 @@
         <v>66</v>
       </c>
       <c r="T15" s="10">
-        <v>938</v>
+        <v>2</v>
       </c>
       <c r="U15" s="11" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="V15" s="10">
         <v>0</v>
@@ -2134,10 +2167,10 @@
         <v>66</v>
       </c>
       <c r="X15" s="10">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="Y15" s="11" t="s">
-        <v>66</v>
+        <v>105</v>
       </c>
       <c r="Z15" s="10">
         <v>0</v>
@@ -2160,13 +2193,13 @@
     </row>
     <row r="16" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C16" s="10">
-        <v>1587</v>
+        <v>69</v>
       </c>
       <c r="D16" s="10">
         <v>0</v>
@@ -2205,10 +2238,10 @@
         <v>66</v>
       </c>
       <c r="P16" s="10">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="Q16" s="11" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="R16" s="10">
         <v>0</v>
@@ -2217,10 +2250,10 @@
         <v>66</v>
       </c>
       <c r="T16" s="10">
-        <v>1540</v>
+        <v>18</v>
       </c>
       <c r="U16" s="11" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="V16" s="10">
         <v>0</v>
@@ -2229,10 +2262,10 @@
         <v>66</v>
       </c>
       <c r="X16" s="10">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Y16" s="11" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="Z16" s="10">
         <v>0</v>
@@ -2255,13 +2288,13 @@
     </row>
     <row r="17" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C17" s="10">
-        <v>1132</v>
+        <v>95</v>
       </c>
       <c r="D17" s="10">
         <v>0</v>
@@ -2300,10 +2333,10 @@
         <v>66</v>
       </c>
       <c r="P17" s="10">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="11" t="s">
-        <v>106</v>
+        <v>66</v>
       </c>
       <c r="R17" s="10">
         <v>0</v>
@@ -2312,10 +2345,10 @@
         <v>66</v>
       </c>
       <c r="T17" s="10">
-        <v>1118</v>
+        <v>34</v>
       </c>
       <c r="U17" s="11" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="V17" s="10">
         <v>0</v>
@@ -2324,10 +2357,10 @@
         <v>66</v>
       </c>
       <c r="X17" s="10">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="Y17" s="11" t="s">
-        <v>66</v>
+        <v>114</v>
       </c>
       <c r="Z17" s="10">
         <v>0</v>
@@ -2350,13 +2383,13 @@
     </row>
     <row r="18" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C18" s="10">
-        <v>338</v>
+        <v>13</v>
       </c>
       <c r="D18" s="10">
         <v>0</v>
@@ -2395,10 +2428,10 @@
         <v>66</v>
       </c>
       <c r="P18" s="10">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="11" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="R18" s="10">
         <v>0</v>
@@ -2407,10 +2440,10 @@
         <v>66</v>
       </c>
       <c r="T18" s="10">
-        <v>331</v>
+        <v>0</v>
       </c>
       <c r="U18" s="11" t="s">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="V18" s="10">
         <v>0</v>
@@ -2419,10 +2452,10 @@
         <v>66</v>
       </c>
       <c r="X18" s="10">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="Y18" s="11" t="s">
-        <v>66</v>
+        <v>117</v>
       </c>
       <c r="Z18" s="10">
         <v>0</v>
@@ -2445,13 +2478,13 @@
     </row>
     <row r="19" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C19" s="10">
-        <v>1524</v>
+        <v>159</v>
       </c>
       <c r="D19" s="10">
         <v>0</v>
@@ -2478,10 +2511,10 @@
         <v>66</v>
       </c>
       <c r="L19" s="10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" s="11" t="s">
-        <v>66</v>
+        <v>120</v>
       </c>
       <c r="N19" s="10">
         <v>0</v>
@@ -2490,10 +2523,10 @@
         <v>66</v>
       </c>
       <c r="P19" s="10">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="Q19" s="11" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="R19" s="10">
         <v>0</v>
@@ -2502,10 +2535,10 @@
         <v>66</v>
       </c>
       <c r="T19" s="10">
-        <v>1501</v>
+        <v>3</v>
       </c>
       <c r="U19" s="11" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="V19" s="10">
         <v>0</v>
@@ -2514,10 +2547,10 @@
         <v>66</v>
       </c>
       <c r="X19" s="10">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="Y19" s="11" t="s">
-        <v>66</v>
+        <v>122</v>
       </c>
       <c r="Z19" s="10">
         <v>0</v>
@@ -2540,13 +2573,13 @@
     </row>
     <row r="20" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C20" s="10">
-        <v>139</v>
+        <v>18</v>
       </c>
       <c r="D20" s="10">
         <v>0</v>
@@ -2573,10 +2606,10 @@
         <v>66</v>
       </c>
       <c r="L20" s="10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M20" s="11" t="s">
-        <v>66</v>
+        <v>125</v>
       </c>
       <c r="N20" s="10">
         <v>0</v>
@@ -2597,10 +2630,10 @@
         <v>66</v>
       </c>
       <c r="T20" s="10">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="U20" s="11" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="V20" s="10">
         <v>0</v>
@@ -2609,10 +2642,10 @@
         <v>66</v>
       </c>
       <c r="X20" s="10">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="Y20" s="11" t="s">
-        <v>66</v>
+        <v>126</v>
       </c>
       <c r="Z20" s="10">
         <v>0</v>
@@ -2635,13 +2668,13 @@
     </row>
     <row r="21" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="C21" s="10">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="D21" s="10">
         <v>0</v>
@@ -2692,10 +2725,10 @@
         <v>66</v>
       </c>
       <c r="T21" s="10">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="U21" s="11" t="s">
-        <v>77</v>
+        <v>129</v>
       </c>
       <c r="V21" s="10">
         <v>0</v>
@@ -2704,10 +2737,10 @@
         <v>66</v>
       </c>
       <c r="X21" s="10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Y21" s="11" t="s">
-        <v>66</v>
+        <v>130</v>
       </c>
       <c r="Z21" s="10">
         <v>0</v>
@@ -2730,13 +2763,13 @@
     </row>
     <row r="22" ht="19" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="C22" s="10">
-        <v>608</v>
+        <v>103</v>
       </c>
       <c r="D22" s="10">
         <v>0</v>
@@ -2775,10 +2808,10 @@
         <v>66</v>
       </c>
       <c r="P22" s="10">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="11" t="s">
-        <v>122</v>
+        <v>66</v>
       </c>
       <c r="R22" s="10">
         <v>0</v>
@@ -2787,10 +2820,10 @@
         <v>66</v>
       </c>
       <c r="T22" s="10">
-        <v>604</v>
+        <v>53</v>
       </c>
       <c r="U22" s="11" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="V22" s="10">
         <v>0</v>
@@ -2799,10 +2832,10 @@
         <v>66</v>
       </c>
       <c r="X22" s="10">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="Y22" s="11" t="s">
-        <v>66</v>
+        <v>134</v>
       </c>
       <c r="Z22" s="10">
         <v>0</v>
@@ -2825,13 +2858,13 @@
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C23" s="13">
-        <v>11782</v>
+        <v>827</v>
       </c>
       <c r="D23" s="13">
         <v>0</v>
@@ -2858,10 +2891,10 @@
         <v>66</v>
       </c>
       <c r="L23" s="13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M23" s="14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N23" s="13">
         <v>0</v>
@@ -2870,10 +2903,10 @@
         <v>66</v>
       </c>
       <c r="P23" s="13">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="Q23" s="14" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="R23" s="13">
         <v>0</v>
@@ -2882,10 +2915,10 @@
         <v>66</v>
       </c>
       <c r="T23" s="13">
-        <v>11632</v>
+        <v>223</v>
       </c>
       <c r="U23" s="14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V23" s="13">
         <v>0</v>
@@ -2894,10 +2927,10 @@
         <v>66</v>
       </c>
       <c r="X23" s="13">
-        <v>0</v>
+        <v>596</v>
       </c>
       <c r="Y23" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="Z23" s="13">
         <v>0</v>

</xml_diff>